<commit_message>
A10 draft: leave Worker Qty blank until confirmed by supervisors
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Nhap_lieu_A10_19-10_den_25-10_NHAP.xlsx
+++ b/loss-time/outputs/Nhap_lieu_A10_19-10_den_25-10_NHAP.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="74">
   <si>
     <t xml:space="preserve">BẢNG NHẬP LIỆU - MACHINING</t>
   </si>
   <si>
-    <t xml:space="preserve">BẢN NHÁP: cột Worker Qty đang lấy theo cột số cuối của báo cáo bảo trì (12 hoặc 24), CẦN XÁC NHẬN đó có phải số công nhân bị ảnh hưởng không. Thứ tự cố định: theo ngày, trong mỗi ngày theo mã P20, P26, P22, A2. Nhập đúng thứ tự cột như form: LossTime Code | Notes | Process | Dept In Charge | From | To | Worker Qty. Nhập xong dòng nào thì đánh dấu X cột "Đã nhập".</t>
+    <t xml:space="preserve">WORKER QTY ĐỂ TRỐNG: chỉ điền SỐ CÔNG NHÂN THẬT đứng máy khi có xác nhận của tổ trưởng khu vực (ghi tên người xác nhận ở cột K). Không dùng cột số cuối (12/24) của báo cáo bảo trì. Thứ tự cố định: theo ngày, trong mỗi ngày theo mã P20, P26, P22, A2. Nhập đúng thứ tự cột như form: LossTime Code | Notes | Process | Dept In Charge | From | To | Worker Qty. Nhập xong dòng nào thì đánh dấu X cột "Đã nhập".</t>
   </si>
   <si>
     <t xml:space="preserve">Ngày (Loss Date)</t>
@@ -60,6 +60,9 @@
     <t xml:space="preserve">Đã nhập</t>
   </si>
   <si>
+    <t xml:space="preserve">Người xác nhận số công nhân</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thứ Hai 19/10/2026: 2 dòng</t>
   </si>
   <si>
@@ -159,10 +162,10 @@
     <t xml:space="preserve">Chênh lệch</t>
   </si>
   <si>
-    <t xml:space="preserve">Cột số cuối (12/24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giờ công = giờ dừng x cột số cuối</t>
+    <t xml:space="preserve">Cột số cuối của báo cáo (chưa rõ nghĩa, KHÔNG dùng làm số công nhân)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giờ công (chưa tính, cần số công nhân thật)</t>
   </si>
   <si>
     <t xml:space="preserve">CNCR02</t>
@@ -235,6 +238,9 @@
   </si>
   <si>
     <t xml:space="preserve">Máy hút chân không</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tổng giờ dừng máy</t>
   </si>
   <si>
     <t xml:space="preserve">Ghi chú: 20/10 máy bơm sơn chuyền UV không có mã máy trong báo cáo. 25/10 là Chủ nhật, báo cáo ghi sự cố máy VC14 khu vực RC (cần xác nhận Raw Cutting có làm hôm đó không). EDB05 ngày 20/10 dừng đến 21:00 (sau giờ tăng ca 20:00).</t>
@@ -326,7 +332,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -351,6 +357,12 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -393,7 +405,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -438,10 +450,18 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -456,6 +476,10 @@
     </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -714,7 +738,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -726,6 +750,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,10 +794,13 @@
       <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="K4" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -783,7 +811,7 @@
       <c r="H5" s="5"/>
       <c r="I5" s="6" t="n">
         <f aca="false">SUM(I6:I7)</f>
-        <v>30.8</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5"/>
     </row>
@@ -792,16 +820,16 @@
         <v>46314</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>0.321527777777778</v>
@@ -809,30 +837,29 @@
       <c r="G6" s="10" t="n">
         <v>0.354166666666667</v>
       </c>
-      <c r="H6" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <f aca="false">(G6-F6)*24*H6</f>
-        <v>18.8</v>
+      <c r="H6" s="11"/>
+      <c r="I6" s="12" t="str">
+        <f aca="false">IF(H6="","",(G6-F6)*24*H6)</f>
+        <v/>
       </c>
       <c r="J6" s="8"/>
+      <c r="K6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>46314</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>16</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0.78125</v>
@@ -840,18 +867,17 @@
       <c r="G7" s="10" t="n">
         <v>0.822916666666667</v>
       </c>
-      <c r="H7" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <f aca="false">(G7-F7)*24*H7</f>
-        <v>12</v>
+      <c r="H7" s="11"/>
+      <c r="I7" s="12" t="str">
+        <f aca="false">IF(H7="","",(G7-F7)*24*H7)</f>
+        <v/>
       </c>
       <c r="J7" s="8"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -862,7 +888,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="6" t="n">
         <f aca="false">SUM(I10:I11)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5"/>
     </row>
@@ -871,16 +897,16 @@
         <v>46315</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0.743055555555556</v>
@@ -888,30 +914,29 @@
       <c r="G10" s="10" t="n">
         <v>0.826388888888889</v>
       </c>
-      <c r="H10" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <f aca="false">(G10-F10)*24*H10</f>
-        <v>24</v>
+      <c r="H10" s="11"/>
+      <c r="I10" s="12" t="str">
+        <f aca="false">IF(H10="","",(G10-F10)*24*H10)</f>
+        <v/>
       </c>
       <c r="J10" s="8"/>
+      <c r="K10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
         <v>46315</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>0.75</v>
@@ -919,18 +944,17 @@
       <c r="G11" s="10" t="n">
         <v>0.875</v>
       </c>
-      <c r="H11" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <f aca="false">(G11-F11)*24*H11</f>
-        <v>36</v>
+      <c r="H11" s="11"/>
+      <c r="I11" s="12" t="str">
+        <f aca="false">IF(H11="","",(G11-F11)*24*H11)</f>
+        <v/>
       </c>
       <c r="J11" s="8"/>
+      <c r="K11" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -941,7 +965,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="6" t="n">
         <f aca="false">SUM(I14:I14)</f>
-        <v>10.2</v>
+        <v>0</v>
       </c>
       <c r="J13" s="5"/>
     </row>
@@ -950,16 +974,16 @@
         <v>46317</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>0.700694444444444</v>
@@ -967,18 +991,17 @@
       <c r="G14" s="10" t="n">
         <v>0.736111111111111</v>
       </c>
-      <c r="H14" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <f aca="false">(G14-F14)*24*H14</f>
-        <v>10.2</v>
+      <c r="H14" s="11"/>
+      <c r="I14" s="12" t="str">
+        <f aca="false">IF(H14="","",(G14-F14)*24*H14)</f>
+        <v/>
       </c>
       <c r="J14" s="8"/>
+      <c r="K14" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -989,7 +1012,7 @@
       <c r="H16" s="5"/>
       <c r="I16" s="6" t="n">
         <f aca="false">SUM(I17:I17)</f>
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="J16" s="5"/>
     </row>
@@ -998,16 +1021,16 @@
         <v>46319</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="10" t="n">
         <v>0.319444444444444</v>
@@ -1015,22 +1038,21 @@
       <c r="G17" s="10" t="n">
         <v>0.328472222222222</v>
       </c>
-      <c r="H17" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <f aca="false">(G17-F17)*24*H17</f>
-        <v>2.6</v>
+      <c r="H17" s="11"/>
+      <c r="I17" s="12" t="str">
+        <f aca="false">IF(H17="","",(G17-F17)*24*H17)</f>
+        <v/>
       </c>
       <c r="J17" s="8"/>
+      <c r="K17" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H19" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I19" s="13" t="n">
+      <c r="H19" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="15" t="n">
         <f aca="false">SUMIF(A5:A18,"&gt;0",I5:I18)</f>
-        <v>103.6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1049,7 +1071,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1061,11 +1083,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1104,10 +1127,13 @@
       <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="K4" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1118,7 +1144,7 @@
       <c r="H5" s="5"/>
       <c r="I5" s="6" t="n">
         <f aca="false">SUM(I6:I6)</f>
-        <v>11.4</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5"/>
     </row>
@@ -1127,16 +1153,16 @@
         <v>46315</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>0.375694444444444</v>
@@ -1144,18 +1170,17 @@
       <c r="G6" s="10" t="n">
         <v>0.415277777777778</v>
       </c>
-      <c r="H6" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <f aca="false">(G6-F6)*24*H6</f>
-        <v>11.4</v>
+      <c r="H6" s="11"/>
+      <c r="I6" s="12" t="str">
+        <f aca="false">IF(H6="","",(G6-F6)*24*H6)</f>
+        <v/>
       </c>
       <c r="J6" s="8"/>
+      <c r="K6" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1166,7 +1191,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="6" t="n">
         <f aca="false">SUM(I9:I9)</f>
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5"/>
     </row>
@@ -1175,16 +1200,16 @@
         <v>46316</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0.774305555555556</v>
@@ -1192,18 +1217,17 @@
       <c r="G9" s="10" t="n">
         <v>0.833333333333333</v>
       </c>
-      <c r="H9" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <f aca="false">(G9-F9)*24*H9</f>
-        <v>17</v>
+      <c r="H9" s="11"/>
+      <c r="I9" s="12" t="str">
+        <f aca="false">IF(H9="","",(G9-F9)*24*H9)</f>
+        <v/>
       </c>
       <c r="J9" s="8"/>
+      <c r="K9" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1214,7 +1238,7 @@
       <c r="H11" s="5"/>
       <c r="I11" s="6" t="n">
         <f aca="false">SUM(I12:I12)</f>
-        <v>20.8</v>
+        <v>0</v>
       </c>
       <c r="J11" s="5"/>
     </row>
@@ -1223,16 +1247,16 @@
         <v>46320</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>0.350694444444444</v>
@@ -1240,22 +1264,21 @@
       <c r="G12" s="10" t="n">
         <v>0.422916666666667</v>
       </c>
-      <c r="H12" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <f aca="false">(G12-F12)*24*H12</f>
-        <v>20.8</v>
+      <c r="H12" s="11"/>
+      <c r="I12" s="12" t="str">
+        <f aca="false">IF(H12="","",(G12-F12)*24*H12)</f>
+        <v/>
       </c>
       <c r="J12" s="8"/>
+      <c r="K12" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H14" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I14" s="13" t="n">
+      <c r="H14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" s="15" t="n">
         <f aca="false">SUMIF(A5:A13,"&gt;0",I5:I13)</f>
-        <v>49.2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1289,46 +1312,46 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1336,16 +1359,16 @@
         <v>46314</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F3" s="10" t="n">
         <v>0.321527777777778</v>
@@ -1356,7 +1379,7 @@
       <c r="H3" s="8" t="n">
         <v>0.78</v>
       </c>
-      <c r="I3" s="15" t="n">
+      <c r="I3" s="17" t="n">
         <f aca="false">(G3-F3)*24</f>
         <v>0.783333333333333</v>
       </c>
@@ -1367,24 +1390,21 @@
       <c r="K3" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="L3" s="11" t="n">
-        <f aca="false">I3*K3</f>
-        <v>18.8</v>
-      </c>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="n">
         <v>46315</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0.375694444444444</v>
@@ -1395,7 +1415,7 @@
       <c r="H4" s="8" t="n">
         <v>0.95</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="17" t="n">
         <f aca="false">(G4-F4)*24</f>
         <v>0.95</v>
       </c>
@@ -1406,26 +1426,23 @@
       <c r="K4" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L4" s="11" t="n">
-        <f aca="false">I4*K4</f>
-        <v>11.4</v>
-      </c>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="n">
         <v>46314</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0.78125</v>
@@ -1436,7 +1453,7 @@
       <c r="H5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="17" t="n">
         <f aca="false">(G5-F5)*24</f>
         <v>1</v>
       </c>
@@ -1447,26 +1464,23 @@
       <c r="K5" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L5" s="11" t="n">
-        <f aca="false">I5*K5</f>
-        <v>12</v>
-      </c>
+      <c r="L5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
         <v>46315</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>0.75</v>
@@ -1477,7 +1491,7 @@
       <c r="H6" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="17" t="n">
         <f aca="false">(G6-F6)*24</f>
         <v>3</v>
       </c>
@@ -1488,26 +1502,23 @@
       <c r="K6" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L6" s="11" t="n">
-        <f aca="false">I6*K6</f>
-        <v>36</v>
-      </c>
+      <c r="L6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>46315</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0.743055555555556</v>
@@ -1518,7 +1529,7 @@
       <c r="H7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="15" t="n">
+      <c r="I7" s="17" t="n">
         <f aca="false">(G7-F7)*24</f>
         <v>2</v>
       </c>
@@ -1529,26 +1540,23 @@
       <c r="K7" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L7" s="11" t="n">
-        <f aca="false">I7*K7</f>
-        <v>24</v>
-      </c>
+      <c r="L7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
         <v>46316</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0.774305555555556</v>
@@ -1559,7 +1567,7 @@
       <c r="H8" s="8" t="n">
         <v>1.42</v>
       </c>
-      <c r="I8" s="15" t="n">
+      <c r="I8" s="17" t="n">
         <f aca="false">(G8-F8)*24</f>
         <v>1.41666666666667</v>
       </c>
@@ -1570,26 +1578,23 @@
       <c r="K8" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L8" s="11" t="n">
-        <f aca="false">I8*K8</f>
-        <v>17</v>
-      </c>
+      <c r="L8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
         <v>46317</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0.700694444444444</v>
@@ -1600,7 +1605,7 @@
       <c r="H9" s="8" t="n">
         <v>0.85</v>
       </c>
-      <c r="I9" s="15" t="n">
+      <c r="I9" s="17" t="n">
         <f aca="false">(G9-F9)*24</f>
         <v>0.85</v>
       </c>
@@ -1611,26 +1616,23 @@
       <c r="K9" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L9" s="11" t="n">
-        <f aca="false">I9*K9</f>
-        <v>10.2</v>
-      </c>
+      <c r="L9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
         <v>46319</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0.319444444444444</v>
@@ -1641,7 +1643,7 @@
       <c r="H10" s="8" t="n">
         <v>0.22</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I10" s="17" t="n">
         <f aca="false">(G10-F10)*24</f>
         <v>0.216666666666667</v>
       </c>
@@ -1652,26 +1654,23 @@
       <c r="K10" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L10" s="11" t="n">
-        <f aca="false">I10*K10</f>
-        <v>2.6</v>
-      </c>
+      <c r="L10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
         <v>46320</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>69</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>68</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>0.350694444444444</v>
@@ -1682,7 +1681,7 @@
       <c r="H11" s="8" t="n">
         <v>1.73</v>
       </c>
-      <c r="I11" s="15" t="n">
+      <c r="I11" s="17" t="n">
         <f aca="false">(G11-F11)*24</f>
         <v>1.73333333333333</v>
       </c>
@@ -1693,23 +1692,20 @@
       <c r="K11" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L11" s="11" t="n">
-        <f aca="false">I11*K11</f>
-        <v>20.8</v>
-      </c>
+      <c r="L11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K12" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="L12" s="13" t="n">
-        <f aca="false">SUM(L3:L11)</f>
-        <v>152.8</v>
+      <c r="H12" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <f aca="false">SUM(I3:I11)</f>
+        <v>11.95</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
-        <v>71</v>
+      <c r="A14" s="19" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A10 draft: add historical worker reference column (reference only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Nhap_lieu_A10_19-10_den_25-10_NHAP.xlsx
+++ b/loss-time/outputs/Nhap_lieu_A10_19-10_den_25-10_NHAP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="84">
   <si>
     <t xml:space="preserve">BẢNG NHẬP LIỆU - MACHINING</t>
   </si>
@@ -168,6 +168,9 @@
     <t xml:space="preserve">Giờ công (chưa tính, cần số công nhân thật)</t>
   </si>
   <si>
+    <t xml:space="preserve">Lịch sử A10 cùng máy (CHỈ THAM KHẢO, không phải số nhập)</t>
+  </si>
+  <si>
     <t xml:space="preserve">CNCR02</t>
   </si>
   <si>
@@ -177,6 +180,9 @@
     <t xml:space="preserve">Lỗi nút bấm</t>
   </si>
   <si>
+    <t xml:space="preserve">Chưa từng có trong A10. Họ CNCR: 2 người (30 lần), 3 người (14 lần)</t>
+  </si>
+  <si>
     <t xml:space="preserve">RC</t>
   </si>
   <si>
@@ -186,6 +192,9 @@
     <t xml:space="preserve">Máy bơm sơn không hoạt động</t>
   </si>
   <si>
+    <t xml:space="preserve">Chưa từng có. Dòng UV khác: 5/6 nhám UV 2 người, 26/6 UVDR01 4 người, 26/6 BECY06 4 người</t>
+  </si>
+  <si>
     <t xml:space="preserve">EDB01</t>
   </si>
   <si>
@@ -195,12 +204,18 @@
     <t xml:space="preserve">Lỗi hộp số</t>
   </si>
   <si>
+    <t xml:space="preserve">Chưa từng có. Họ EDB: 2 người (3 lần), 3 người (1 lần)</t>
+  </si>
+  <si>
     <t xml:space="preserve">EDB05</t>
   </si>
   <si>
     <t xml:space="preserve">Lỗi nồi keo</t>
   </si>
   <si>
+    <t xml:space="preserve">1 lần: 25/6 13:50-14:30, 3 người</t>
+  </si>
+  <si>
     <t xml:space="preserve">CNCR09</t>
   </si>
   <si>
@@ -210,6 +225,9 @@
     <t xml:space="preserve">Lỗi trục không quay</t>
   </si>
   <si>
+    <t xml:space="preserve">Chưa từng có. Máy chép hình tròn 60-0041 từng ghi 2 người (khác loại)</t>
+  </si>
+  <si>
     <t xml:space="preserve">VEC04</t>
   </si>
   <si>
@@ -219,12 +237,18 @@
     <t xml:space="preserve">Máy tự cắt</t>
   </si>
   <si>
+    <t xml:space="preserve">4 lần (30/12, 20/1, 23/1, 30/7): đều 2 người</t>
+  </si>
+  <si>
     <t xml:space="preserve">CNCR20</t>
   </si>
   <si>
     <t xml:space="preserve">Gãy giá đỡ dây điện</t>
   </si>
   <si>
+    <t xml:space="preserve">3 dòng: 1/6 hai lần 2 người; 4/4 cả ngày 4 người (dòng bất thường)</t>
+  </si>
+  <si>
     <t xml:space="preserve">CNCR11</t>
   </si>
   <si>
@@ -234,10 +258,16 @@
     <t xml:space="preserve">Lỗi hút chân không</t>
   </si>
   <si>
+    <t xml:space="preserve">1 lần: 9/4 Hogmag piton hút bụi, 2 người</t>
+  </si>
+  <si>
     <t xml:space="preserve">VC14</t>
   </si>
   <si>
     <t xml:space="preserve">Máy hút chân không</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa từng có. Máy hút chân không CNCR14 từng ghi 3 người</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng giờ dừng máy</t>
@@ -258,7 +288,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +355,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="11"/>
       <name val="Times New Roman"/>
@@ -405,7 +442,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -478,11 +515,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -512,7 +553,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
@@ -1297,7 +1338,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
@@ -1309,6 +1350,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1353,6 +1395,9 @@
       <c r="L2" s="3" t="s">
         <v>47</v>
       </c>
+      <c r="M2" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="n">
@@ -1362,13 +1407,13 @@
         <v>16</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F3" s="10" t="n">
         <v>0.321527777777778</v>
@@ -1391,20 +1436,23 @@
         <v>24</v>
       </c>
       <c r="L3" s="12"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M3" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="n">
         <v>46315</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0.375694444444444</v>
@@ -1427,6 +1475,9 @@
         <v>12</v>
       </c>
       <c r="L4" s="12"/>
+      <c r="M4" s="18" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="n">
@@ -1436,13 +1487,13 @@
         <v>16</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0.78125</v>
@@ -1465,6 +1516,9 @@
         <v>12</v>
       </c>
       <c r="L5" s="12"/>
+      <c r="M5" s="18" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
@@ -1474,13 +1528,13 @@
         <v>16</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>0.75</v>
@@ -1503,8 +1557,11 @@
         <v>12</v>
       </c>
       <c r="L6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M6" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>46315</v>
       </c>
@@ -1512,13 +1569,13 @@
         <v>16</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0.743055555555556</v>
@@ -1541,22 +1598,25 @@
         <v>12</v>
       </c>
       <c r="L7" s="12"/>
+      <c r="M7" s="18" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
         <v>46316</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0.774305555555556</v>
@@ -1579,6 +1639,9 @@
         <v>12</v>
       </c>
       <c r="L8" s="12"/>
+      <c r="M8" s="18" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
@@ -1588,13 +1651,13 @@
         <v>16</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0.700694444444444</v>
@@ -1617,6 +1680,9 @@
         <v>12</v>
       </c>
       <c r="L9" s="12"/>
+      <c r="M9" s="18" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
@@ -1626,13 +1692,13 @@
         <v>16</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0.319444444444444</v>
@@ -1655,22 +1721,25 @@
         <v>12</v>
       </c>
       <c r="L10" s="12"/>
+      <c r="M10" s="18" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
         <v>46320</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>0.350694444444444</v>
@@ -1693,19 +1762,22 @@
         <v>12</v>
       </c>
       <c r="L11" s="12"/>
+      <c r="M11" s="18" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H12" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="18" t="n">
+        <v>82</v>
+      </c>
+      <c r="I12" s="19" t="n">
         <f aca="false">SUM(I3:I11)</f>
         <v>11.95</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>73</v>
+      <c r="A14" s="20" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>